<commit_message>
Update: Adição de métricas de avaliação dos Modelos treinados
</commit_message>
<xml_diff>
--- a/docs/Available Models.xlsx
+++ b/docs/Available Models.xlsx
@@ -5,18 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guilherme\Desktop\6º Semestre\TCC\Modelos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guilherme\Desktop\6º Semestre\TCC\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7111C93A-6C80-4A4D-BA46-B907913D5A55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41E41B18-11BC-4DF3-A937-D2BD6F58BB7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{69908BCD-CF23-4C8B-B737-0A5881F10D2A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{69908BCD-CF23-4C8B-B737-0A5881F10D2A}"/>
   </bookViews>
   <sheets>
-    <sheet name="Models" sheetId="1" r:id="rId1"/>
+    <sheet name="Hardware specifications" sheetId="2" r:id="rId1"/>
+    <sheet name="Models Keras" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Models!$C$6:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Models Keras'!$C$6:$J$6</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="207">
   <si>
     <t>50.2M</t>
   </si>
@@ -642,13 +643,34 @@
   </si>
   <si>
     <t>350.1M</t>
+  </si>
+  <si>
+    <t>13th Gen Intel(R) Core(TM) i5-13420H (12 CPUs), ~2.1GHz</t>
+  </si>
+  <si>
+    <t>RAM</t>
+  </si>
+  <si>
+    <t>GPU</t>
+  </si>
+  <si>
+    <t>Intel(R) UHD Graphics &amp; NVIDIA GeForce RTX 3050 6GB Laptop GPU</t>
+  </si>
+  <si>
+    <t>CONFIGS COMPUTER</t>
+  </si>
+  <si>
+    <t>PROCESSOR:</t>
+  </si>
+  <si>
+    <t>16 GB DDR5, 5200 MT/s</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -691,6 +713,25 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1B1B1B"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -706,7 +747,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -950,12 +991,70 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1019,6 +1118,25 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1354,20 +1472,71 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D395078B-3005-48DD-AFE7-E993F1F07A92}">
+  <dimension ref="B2:C6"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" style="22"/>
+    <col min="2" max="2" width="15.77734375" style="22" customWidth="1"/>
+    <col min="3" max="3" width="70.77734375" style="22" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="22"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:3" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="C3" s="24"/>
+    </row>
+    <row r="4" spans="2:3" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="25" t="s">
+        <v>205</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="26" t="s">
+        <v>201</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="27" t="s">
+        <v>202</v>
+      </c>
+      <c r="C6" s="28" t="s">
+        <v>203</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B3:C3"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA24E35D-486A-43A4-B893-5CDB6FE982A9}">
   <dimension ref="C2:K121"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="60.7109375" customWidth="1"/>
-    <col min="4" max="8" width="22.7109375" customWidth="1"/>
-    <col min="9" max="10" width="24.7109375" customWidth="1"/>
+    <col min="3" max="3" width="60.6640625" customWidth="1"/>
+    <col min="4" max="8" width="22.6640625" customWidth="1"/>
+    <col min="9" max="10" width="24.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="3:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="3:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C4" s="16" t="s">
         <v>9</v>
       </c>
@@ -1380,7 +1549,7 @@
       <c r="J4" s="18"/>
       <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="3:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C5" s="19"/>
       <c r="D5" s="20"/>
       <c r="E5" s="20"/>
@@ -1391,7 +1560,7 @@
       <c r="J5" s="21"/>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="3:11" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:11" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
@@ -1417,7 +1586,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="3:11" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:11" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C7" s="5" t="s">
         <v>18</v>
       </c>
@@ -1443,7 +1612,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C8" s="6" t="s">
         <v>24</v>
       </c>
@@ -1469,7 +1638,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C9" s="6" t="s">
         <v>29</v>
       </c>
@@ -1495,7 +1664,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C10" s="6" t="s">
         <v>33</v>
       </c>
@@ -1521,7 +1690,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C11" s="6" t="s">
         <v>38</v>
       </c>
@@ -1547,7 +1716,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C12" s="6" t="s">
         <v>42</v>
       </c>
@@ -1573,7 +1742,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C13" s="6" t="s">
         <v>48</v>
       </c>
@@ -1599,7 +1768,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C14" s="6" t="s">
         <v>53</v>
       </c>
@@ -1625,7 +1794,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C15" s="6" t="s">
         <v>59</v>
       </c>
@@ -1651,7 +1820,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="16" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:11" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C16" s="6" t="s">
         <v>64</v>
       </c>
@@ -1677,7 +1846,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="17" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C17" s="6" t="s">
         <v>70</v>
       </c>
@@ -1703,7 +1872,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C18" s="6" t="s">
         <v>76</v>
       </c>
@@ -1729,7 +1898,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="19" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C19" s="6" t="s">
         <v>81</v>
       </c>
@@ -1755,7 +1924,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="20" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C20" s="6" t="s">
         <v>84</v>
       </c>
@@ -1781,7 +1950,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="21" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C21" s="6" t="s">
         <v>89</v>
       </c>
@@ -1807,7 +1976,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="22" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C22" s="6" t="s">
         <v>95</v>
       </c>
@@ -1833,7 +2002,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="23" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C23" s="6" t="s">
         <v>101</v>
       </c>
@@ -1859,7 +2028,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C24" s="6" t="s">
         <v>105</v>
       </c>
@@ -1885,7 +2054,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="25" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C25" s="6" t="s">
         <v>111</v>
       </c>
@@ -1911,7 +2080,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="26" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C26" s="6" t="s">
         <v>116</v>
       </c>
@@ -1937,7 +2106,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="27" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C27" s="6" t="s">
         <v>122</v>
       </c>
@@ -1963,7 +2132,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C28" s="6" t="s">
         <v>126</v>
       </c>
@@ -1989,7 +2158,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="29" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C29" s="6" t="s">
         <v>132</v>
       </c>
@@ -2015,7 +2184,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="30" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C30" s="6" t="s">
         <v>138</v>
       </c>
@@ -2041,7 +2210,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="31" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C31" s="6" t="s">
         <v>144</v>
       </c>
@@ -2067,7 +2236,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="32" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C32" s="6" t="s">
         <v>150</v>
       </c>
@@ -2093,7 +2262,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="33" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C33" s="6" t="s">
         <v>156</v>
       </c>
@@ -2119,7 +2288,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="34" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C34" s="6" t="s">
         <v>161</v>
       </c>
@@ -2145,7 +2314,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="35" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C35" s="6" t="s">
         <v>165</v>
       </c>
@@ -2171,7 +2340,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="36" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C36" s="6" t="s">
         <v>169</v>
       </c>
@@ -2197,7 +2366,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="37" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C37" s="6" t="s">
         <v>173</v>
       </c>
@@ -2223,7 +2392,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="38" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C38" s="6" t="s">
         <v>176</v>
       </c>
@@ -2249,7 +2418,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="39" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C39" s="6" t="s">
         <v>180</v>
       </c>
@@ -2275,7 +2444,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="40" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C40" s="6" t="s">
         <v>184</v>
       </c>
@@ -2301,7 +2470,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="41" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C41" s="6" t="s">
         <v>187</v>
       </c>
@@ -2327,7 +2496,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="42" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C42" s="6" t="s">
         <v>190</v>
       </c>
@@ -2353,7 +2522,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="43" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C43" s="6" t="s">
         <v>193</v>
       </c>
@@ -2379,7 +2548,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="44" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="3:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C44" s="7" t="s">
         <v>197</v>
       </c>
@@ -2405,83 +2574,83 @@
         <v>160</v>
       </c>
     </row>
-    <row r="45" spans="3:10" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="3:10" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="3:10" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="3:10" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="70" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="72" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="73" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="75" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="76" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="77" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="78" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="79" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="80" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="81" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="82" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="83" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="84" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="85" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="86" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="87" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="88" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="89" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="90" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="91" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="92" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="93" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="94" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="95" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="96" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="97" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="98" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="99" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="100" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="101" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="102" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="103" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="104" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="105" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="106" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="107" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="108" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="109" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="110" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="111" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="112" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="113" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="114" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="115" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="116" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="117" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="118" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="119" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="120" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="121" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="3:10" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="46" spans="3:10" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="3:10" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="48" spans="3:10" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="49" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="50" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="51" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="52" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="53" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="54" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="55" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="57" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="58" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="59" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="60" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="61" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="62" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="63" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="64" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="65" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="66" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="67" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="68" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="69" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="70" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="71" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="72" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="73" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="74" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="75" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="76" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="77" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="78" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="79" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="80" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="81" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="82" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="83" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="84" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="85" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="86" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="87" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="88" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="89" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="90" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="91" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="92" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="93" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="94" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="95" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="96" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="97" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="98" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="99" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="100" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="101" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="102" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="103" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="104" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="105" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="106" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="107" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="108" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="109" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="110" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="111" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="112" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="113" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="114" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="115" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="116" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="117" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="118" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="119" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="120" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="121" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <autoFilter ref="C6:J6" xr:uid="{AA24E35D-486A-43A4-B893-5CDB6FE982A9}"/>
   <mergeCells count="1">

</xml_diff>